<commit_message>
batch method improved to output plots and accept .csv input files
</commit_message>
<xml_diff>
--- a/inst/extdata/7843_1ng_4.xlsx
+++ b/inst/extdata/7843_1ng_4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\oslo\share\342-Projets_BGE\342.1-EDyP\342.1.1-Projets\342.1.1.82-PSAQ+1\PSAQ+1 Manips\Résultats\8e manip gamme 2.0 29-06-2023\20250922_Verif code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Local\bruley\Dev\rPSAQ\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{254D1E52-3499-47B9-AEFC-05365050C075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{528F3F6B-94DA-46EA-8F58-AF3F32C6143A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{F8D7A8B3-61D4-441F-A8FB-BF1E51DA9C75}"/>
+    <workbookView xWindow="-28920" yWindow="-660" windowWidth="29040" windowHeight="15720" xr2:uid="{F8D7A8B3-61D4-441F-A8FB-BF1E51DA9C75}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -515,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE2D2852-24C8-4EC6-A230-080C40F4153A}">
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="52.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="5" bestFit="1" customWidth="1"/>
@@ -531,7 +534,7 @@
     <col min="11" max="11" width="27.140625" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -566,7 +569,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
@@ -599,7 +602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>27</v>
       </c>
@@ -631,9 +634,8 @@
       <c r="K3" s="3">
         <v>3877.1660000000002</v>
       </c>
-      <c r="L3" s="2"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
@@ -666,7 +668,7 @@
         <v>30504.828000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
@@ -699,7 +701,7 @@
         <v>44758.440999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -732,7 +734,7 @@
         <v>43974.629000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
@@ -765,7 +767,7 @@
         <v>34532.211000000003</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -797,9 +799,8 @@
       <c r="K8" s="3">
         <v>44788.608999999997</v>
       </c>
-      <c r="L8" s="2"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
@@ -832,7 +833,7 @@
         <v>24615.982</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>27</v>
       </c>
@@ -865,7 +866,7 @@
         <v>68603.531000000003</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
@@ -898,7 +899,7 @@
         <v>11417.907999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -931,7 +932,7 @@
         <v>11616.341</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
@@ -964,7 +965,7 @@
         <v>13315.862999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>27</v>
       </c>
@@ -997,7 +998,7 @@
         <v>2529.1</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>27</v>
       </c>
@@ -1030,7 +1031,7 @@
         <v>10409.045</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>27</v>
       </c>

</xml_diff>